<commit_message>
updated rule description and test data
</commit_message>
<xml_diff>
--- a/rules/CORE-000361/negative/01/data/unit-test-coreid-CG0035-negative-1.xlsx
+++ b/rules/CORE-000361/negative/01/data/unit-test-coreid-CG0035-negative-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JanakiRaman\CORE\Rule_Authoring\core-contributor\rules\CORE-000361\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17DEE6D5-D45F-4C3A-91B1-F8B391AE0EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{472B9801-B24D-468A-AC98-26C13E7B1762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -19,12 +19,16 @@
     <sheet name="sv.xpt" sheetId="4" r:id="rId4"/>
     <sheet name="tv.xpt" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">sv.xpt!$A$1:$J$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">tv.xpt!$A$1:$H$33</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="174">
   <si>
     <t>Product</t>
   </si>
@@ -631,7 +635,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -655,8 +659,20 @@
     <xf numFmtId="49" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -988,6 +1004,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="11.54296875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -1020,12 +1039,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.7265625" customWidth="1"/>
+    <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.1796875" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="6" max="6" width="14.453125" style="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -1044,12 +1064,12 @@
       <c r="E1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="12" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
       <c r="B2" t="s">
@@ -1058,18 +1078,18 @@
       <c r="C2" t="s">
         <v>172</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="9">
         <v>34</v>
       </c>
       <c r="E2" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="10" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3">
+      <c r="A3" s="9">
         <v>2</v>
       </c>
       <c r="B3" t="s">
@@ -1078,18 +1098,18 @@
       <c r="C3" t="s">
         <v>172</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="9">
         <v>35</v>
       </c>
       <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="10" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4">
+      <c r="A4" s="9">
         <v>3</v>
       </c>
       <c r="B4" t="s">
@@ -1098,19 +1118,19 @@
       <c r="C4" t="s">
         <v>172</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="9">
         <v>36</v>
       </c>
       <c r="E4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="10" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>1</v>
+      <c r="A5" s="9">
+        <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
@@ -1118,19 +1138,19 @@
       <c r="C5" t="s">
         <v>172</v>
       </c>
-      <c r="D5">
-        <v>34</v>
+      <c r="D5" s="9">
+        <v>5</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="9">
-        <v>100</v>
+        <v>20</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>2</v>
+      <c r="A6" s="9">
+        <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
@@ -1138,19 +1158,19 @@
       <c r="C6" t="s">
         <v>172</v>
       </c>
-      <c r="D6">
-        <v>35</v>
+      <c r="D6" s="9">
+        <v>6</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="9">
-        <v>200</v>
+        <v>20</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>3</v>
+      <c r="A7" s="9">
+        <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
@@ -1158,13 +1178,133 @@
       <c r="C7" t="s">
         <v>172</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="9">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="9">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>172</v>
+      </c>
+      <c r="D8" s="9">
+        <v>34</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="9">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>172</v>
+      </c>
+      <c r="D9" s="9">
+        <v>35</v>
+      </c>
+      <c r="E9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="10">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="9">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>172</v>
+      </c>
+      <c r="D10" s="9">
         <v>36</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E10" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F10" s="10">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="9">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>172</v>
+      </c>
+      <c r="D11" s="9">
+        <v>5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="13">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="9">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>172</v>
+      </c>
+      <c r="D12" s="9">
+        <v>6</v>
+      </c>
+      <c r="E12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="10">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="9">
+        <v>6</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>172</v>
+      </c>
+      <c r="D13" s="9">
+        <v>7</v>
+      </c>
+      <c r="E13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="11">
         <v>300</v>
       </c>
     </row>
@@ -1177,6 +1317,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J62"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="3" max="3" width="18.26953125" customWidth="1"/>
+    <col min="4" max="4" width="14.08984375" customWidth="1"/>
+    <col min="5" max="5" width="18.6328125" customWidth="1"/>
+    <col min="6" max="6" width="9.90625" customWidth="1"/>
+    <col min="7" max="7" width="13.90625" customWidth="1"/>
+    <col min="8" max="8" width="20.1796875" customWidth="1"/>
+    <col min="9" max="9" width="22.1796875" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
@@ -1316,10 +1467,10 @@
       <c r="C5" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="8">
         <v>100</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="8" t="s">
         <v>41</v>
       </c>
       <c r="F5" s="7">
@@ -1345,10 +1496,10 @@
       <c r="C6" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="8">
         <v>200</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="8" t="s">
         <v>44</v>
       </c>
       <c r="F6" s="7">
@@ -1374,10 +1525,10 @@
       <c r="C7" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="8">
         <v>300</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="8" t="s">
         <v>47</v>
       </c>
       <c r="F7" s="7">
@@ -2989,6 +3140,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J62" xr:uid="{00000000-0001-0000-0300-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2997,6 +3149,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="3" max="3" width="15.1796875" customWidth="1"/>
+    <col min="4" max="4" width="19.7265625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
@@ -3686,6 +3843,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H33" xr:uid="{00000000-0001-0000-0400-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>